<commit_message>
Bump to 7.21.5: bigger text on the Daily Lineup Excel
Bumped every font used by the "ACTUAL (new template )" sheet in
lineup-template.xlsx by 2pt (12->14, 16->18, 20->22, etc.) - Carlos
said the printed sheet was hard to read. Only the sz attribute on the
21 font entries actually referenced by that sheet's cells changed;
bold/italic/underline/color/name, borders, merges, formulas, the
portrait+fit-to-page setup and the centered/no-highlight formatting
from 7.21.4 are all untouched. Sheet still auto-fits to one page
regardless of font size since fitToWidth/fitToHeight stay at 1.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/lineup-template.xlsx
+++ b/lineup-template.xlsx
@@ -503,7 +503,7 @@
     </font>
     <font>
       <i/>
-      <sz val="11"/>
+      <sz val="13"/>
       <color theme="1"/>
       <name val="Calibri"/>
       <family val="2"/>
@@ -512,7 +512,7 @@
     <font>
       <b/>
       <i/>
-      <sz val="16"/>
+      <sz val="18"/>
       <color theme="1"/>
       <name val="Calibri"/>
       <family val="2"/>
@@ -520,14 +520,14 @@
     </font>
     <font>
       <b/>
-      <sz val="16"/>
+      <sz val="18"/>
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
     </font>
     <font>
       <i/>
-      <sz val="16"/>
+      <sz val="18"/>
       <color theme="1"/>
       <name val="Calibri"/>
       <family val="2"/>
@@ -535,67 +535,27 @@
     </font>
     <font>
       <i/>
-      <sz val="16"/>
+      <sz val="18"/>
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
     </font>
     <font>
       <i/>
-      <sz val="12"/>
+      <sz val="14"/>
       <color theme="1"/>
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
     </font>
     <font>
-      <sz val="16"/>
+      <sz val="18"/>
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
     </font>
     <font>
       <b/>
-      <sz val="14"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="11"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="12"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="20"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="14"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="12"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <u/>
       <sz val="16"/>
       <name val="Calibri"/>
       <family val="2"/>
@@ -609,7 +569,47 @@
       <scheme val="minor"/>
     </font>
     <font>
-      <sz val="10"/>
+      <b/>
+      <sz val="14"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="22"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="16"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="14"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <u/>
+      <sz val="18"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="15"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="12"/>
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -633,7 +633,7 @@
     </font>
     <font>
       <b/>
-      <sz val="16"/>
+      <sz val="18"/>
       <color theme="1"/>
       <name val="Calibri"/>
       <family val="2"/>
@@ -641,7 +641,7 @@
     </font>
     <font>
       <b/>
-      <sz val="12"/>
+      <sz val="14"/>
       <color theme="1"/>
       <name val="Calibri"/>
       <family val="2"/>
@@ -649,14 +649,14 @@
     </font>
     <font>
       <b/>
-      <sz val="16"/>
+      <sz val="18"/>
       <color theme="0"/>
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
     </font>
     <font>
-      <sz val="12"/>
+      <sz val="14"/>
       <color theme="1"/>
       <name val="Calibri"/>
       <family val="2"/>
@@ -665,7 +665,7 @@
     <font>
       <b/>
       <i/>
-      <sz val="14"/>
+      <sz val="16"/>
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -753,7 +753,7 @@
     </font>
     <font>
       <i/>
-      <sz val="14"/>
+      <sz val="16"/>
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>

</xml_diff>

<commit_message>
Bump to 7.21.6: wider GRA name box + shortened names on the Daily Lineup
Carlos hand-writes the room total and check-out total on either side
of the GRA's name on the printed sheet, so the name box was too tight:

- Widened columns E and I (the GRA name grid, rows 35-45 plus the 3
  floater slots) from ~15/16 to ~20/21 - more blank margin either side
  of the printed name for his handwriting.
- Added dlShortName(): GRA and floater names now export as "First L."
  (e.g. "Maria Aguilar" -> "Maria A") instead of the full name, freeing
  up even more room inside the wider box. Scoped to just that grid -
  coordinators, supervisors, house attendants, lobby and night crews
  still print in full.

Column widths patched via the same targeted XML surgery as the prior
template edits; dlShortName lives in the app code (index.html), not
the template, since it only affects what gets written into the cells,
not their formatting.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/lineup-template.xlsx
+++ b/lineup-template.xlsx
@@ -3054,11 +3054,11 @@
     <col min="2" max="2" width="14.28515625" style="9" customWidth="1"/>
     <col min="3" max="3" width="13.140625" style="9" customWidth="1"/>
     <col min="4" max="4" width="12.7109375" style="9" customWidth="1"/>
-    <col min="5" max="5" width="15.140625" style="9" customWidth="1"/>
+    <col min="5" max="5" width="20.140625" style="9" customWidth="1"/>
     <col min="6" max="6" width="13" style="9" customWidth="1"/>
     <col min="7" max="7" width="12.7109375" style="9" customWidth="1"/>
     <col min="8" max="8" width="2.140625" style="9" customWidth="1"/>
-    <col min="9" max="9" width="16.140625" style="9" customWidth="1"/>
+    <col min="9" max="9" width="21.140625" style="9" customWidth="1"/>
     <col min="10" max="10" width="16.42578125" style="9" customWidth="1"/>
     <col min="11" max="11" width="61.7109375" style="9" customWidth="1"/>
     <col min="12" max="12" width="1" style="9" customWidth="1"/>

</xml_diff>